<commit_message>
Reformatacao pos recuperacao lista inicial
Reformatacao apos recuperacao da lista inicial, nao formatada e vazia
</commit_message>
<xml_diff>
--- a/PastaDocsEngenhariaSw/ListaDeRequisitosSiEstacionamento.xlsx
+++ b/PastaDocsEngenhariaSw/ListaDeRequisitosSiEstacionamento.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\renat\Downloads\Projetos2SIR-2026\Projetos2SIPG\PastaDocsEngenhariaSw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C28C599-CDDD-4B53-A5B9-9CEE35A8A8B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1E45BA9-B7E2-4263-9426-06E1C6721D77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -66,7 +66,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -89,6 +89,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="5" tint="-0.499984740745262"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -99,13 +107,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="3" tint="-0.249977111117893"/>
+        <fgColor theme="5" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.39997558519241921"/>
+        <fgColor theme="5" tint="-0.249977111117893"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -140,9 +148,9 @@
   <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -431,15 +439,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="4"/>
+      <c r="B2" s="2"/>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">

</xml_diff>